<commit_message>
feat: enable cold-recipient WhatsApp broadcast templates and sync latest live database backup
</commit_message>
<xml_diff>
--- a/data/teams_export.xlsx
+++ b/data/teams_export.xlsx
@@ -397,41 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF6"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" customWidth="1"/>
-    <col min="6" max="6" width="48.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="48.83203125" customWidth="1"/>
-    <col min="9" max="9" width="48.83203125" customWidth="1"/>
-    <col min="10" max="10" width="48.83203125" customWidth="1"/>
-    <col min="11" max="11" width="48.83203125" customWidth="1"/>
-    <col min="12" max="12" width="48.83203125" customWidth="1"/>
-    <col min="13" max="13" width="16.83203125" customWidth="1"/>
-    <col min="14" max="14" width="16.83203125" customWidth="1"/>
-    <col min="15" max="15" width="19.83203125" customWidth="1"/>
-    <col min="16" max="16" width="16.83203125" customWidth="1"/>
-    <col min="17" max="17" width="16.83203125" customWidth="1"/>
-    <col min="18" max="18" width="19.83203125" customWidth="1"/>
-    <col min="19" max="19" width="21.83203125" customWidth="1"/>
-    <col min="20" max="20" width="16.83203125" customWidth="1"/>
-    <col min="21" max="21" width="19.83203125" customWidth="1"/>
-    <col min="22" max="22" width="16.83203125" customWidth="1"/>
-    <col min="23" max="23" width="16.83203125" customWidth="1"/>
-    <col min="24" max="24" width="19.83203125" customWidth="1"/>
-    <col min="25" max="25" width="16.83203125" customWidth="1"/>
-    <col min="26" max="26" width="16.83203125" customWidth="1"/>
-    <col min="27" max="27" width="19.83203125" customWidth="1"/>
-    <col min="28" max="28" width="16.83203125" customWidth="1"/>
-    <col min="29" max="29" width="16.83203125" customWidth="1"/>
-    <col min="30" max="30" width="19.83203125" customWidth="1"/>
-    <col min="31" max="31" width="15.83203125" customWidth="1"/>
-    <col min="32" max="32" width="25.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:AF4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -533,58 +499,58 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CSEEXPO-2026-0004</v>
+        <v>CSEEXPO-2026-0003</v>
       </c>
       <c r="B2" t="str">
-        <v>GreenGrid Micro</v>
+        <v>Techora</v>
       </c>
       <c r="C2" t="str">
-        <v>Ananya Reddy</v>
+        <v>Madhu Sree</v>
       </c>
       <c r="D2" t="str">
-        <v>+919876543213</v>
+        <v>+919025896972</v>
       </c>
       <c r="E2" t="str">
-        <v>ananya.reddy@gmail.com</v>
+        <v>madhusreemanokaran@gmail.com</v>
       </c>
       <c r="F2" t="str">
-        <v>Autonomous Campus Renewable Microgrid Load Balancer</v>
+        <v>Gridguard Ai</v>
       </c>
       <c r="G2" t="str">
-        <v>Smart Campus</v>
+        <v>Artificial Intelligence</v>
       </c>
       <c r="H2" t="str">
-        <v>Campuses experience erratic power distribution and waste diesel generator fuel during peak hours.</v>
+        <v>Gridguard Ai in Lt line and automatic emergency shutdown</v>
       </c>
       <c r="I2" t="str">
-        <v>An intelligent power controller utilizing deep Q-learning to dynamically shift heavy HVAC loads to solar battery banks.</v>
+        <v>Using Sensors like temperature,voltage we can find the status of Lt line</v>
       </c>
       <c r="J2" t="str">
-        <v>Next.js, PyTorch, Node-RED, Modbus TCP, TimescaleDB</v>
+        <v>Python Flask</v>
       </c>
       <c r="K2" t="str">
-        <v>Arduino Mega 2560, ACS712 Current Sensors, ZMPT101B Voltage Sensors, Solid State Relays (40A)</v>
+        <v>Lora Module</v>
       </c>
       <c r="L2" t="str">
-        <v>18% reduction in grid electricity consumption.</v>
+        <v/>
       </c>
       <c r="M2" t="str">
-        <v>Ananya Reddy</v>
+        <v>Madhu Sree</v>
       </c>
       <c r="N2" t="str">
-        <v>4th Year</v>
+        <v>3rd Year</v>
       </c>
       <c r="O2" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="P2" t="str">
-        <v>Ishaan Pillai</v>
+        <v>Gracy</v>
       </c>
       <c r="Q2" t="str">
-        <v>4th Year</v>
+        <v>3rd Year</v>
       </c>
       <c r="R2" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="S2" t="str">
         <v/>
@@ -626,7 +592,7 @@
         <v>SUBMITTED</v>
       </c>
       <c r="AF2" t="str">
-        <v>28 Sept 2026, 05:13 am</v>
+        <v>2026-09-29T00:23:54.151Z</v>
       </c>
     </row>
     <row r="3">
@@ -721,84 +687,84 @@
         <v/>
       </c>
       <c r="AE3" t="str">
-        <v>UNDER_REVIEW</v>
+        <v>REJECTED</v>
       </c>
       <c r="AF3" t="str">
-        <v>27 Sept 2026, 05:13 am</v>
+        <v>2026-09-26T23:59:34.774Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>CSEEXPO-2026-0001</v>
+        <v>CSEEXPO-2026-0005</v>
       </c>
       <c r="B4" t="str">
-        <v>AgriSense IoT</v>
+        <v>SafeStream AI</v>
       </c>
       <c r="C4" t="str">
-        <v>Aarav Sharma</v>
+        <v>Vikram Singh</v>
       </c>
       <c r="D4" t="str">
-        <v>+919876543210</v>
+        <v>+919876543214</v>
       </c>
       <c r="E4" t="str">
-        <v>aarav.sharma@gmail.com</v>
+        <v>vikram.singh@gmail.com</v>
       </c>
       <c r="F4" t="str">
-        <v>Precision Soil Health &amp; Automated Irrigation System</v>
+        <v>Vision-Based Industrial Machine Safety Interlock</v>
       </c>
       <c r="G4" t="str">
-        <v>Agriculture</v>
+        <v>Artificial Intelligence</v>
       </c>
       <c r="H4" t="str">
-        <v>Traditional farming leads to 40% water wastage and excessive chemical fertilizer usage due to lack of real-time soil nutrient and moisture data.</v>
+        <v>Accidents at mechanical presses occur when operators bypass safety light curtains during shifts.</v>
       </c>
       <c r="I4" t="str">
-        <v>An edge-AI enabled smart telemetry system with multi-depth soil probes, automated solenoid irrigation valves, and a React Native dashboard.</v>
+        <v>Stereo-vision edge module tracking operator hands, predicting trajectory, and triggering electronic emergency brakes in 40ms.</v>
       </c>
       <c r="J4" t="str">
-        <v>Next.js, Python, Flask, TensorFlow Lite, MQTT, InfluxDB</v>
+        <v>C++, OpenCV, CUDA, TensorRT, Electron Dashboard</v>
       </c>
       <c r="K4" t="str">
-        <v>ESP32 DevKit, Capacitive Soil Moisture Sensors, NPK Soil Sensor, 12V Solenoid Valves, LoRa Ra-02 Module</v>
+        <v>NVIDIA Jetson Orin Nano, Dual Global Shutter CSI Cameras, Optocoupler Relay Isolation Board</v>
       </c>
       <c r="L4" t="str">
-        <v>35% water savings and early detection of nutrient deficiencies.</v>
+        <v>Zero false negatives in safety hazard classification.</v>
       </c>
       <c r="M4" t="str">
-        <v>Aarav Sharma</v>
+        <v>Vikram Singh</v>
       </c>
       <c r="N4" t="str">
         <v>3rd Year</v>
       </c>
       <c r="O4" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="P4" t="str">
-        <v>Bhavya Gupta</v>
+        <v>Jaya Prakash</v>
       </c>
       <c r="Q4" t="str">
         <v>3rd Year</v>
       </c>
       <c r="R4" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="S4" t="str">
-        <v>Chirag Singhal</v>
+        <v>Karan Malhotra</v>
       </c>
       <c r="T4" t="str">
         <v>3rd Year</v>
       </c>
       <c r="U4" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="V4" t="str">
-        <v>Deepak Joshi</v>
+        <v/>
       </c>
       <c r="W4" t="str">
-        <v>3rd Year</v>
+        <v/>
       </c>
       <c r="X4" t="str">
-        <v>A</v>
+        <v/>
       </c>
       <c r="Y4" t="str">
         <v/>
@@ -822,208 +788,12 @@
         <v>SHORTLISTED</v>
       </c>
       <c r="AF4" t="str">
-        <v>26 Sept 2026, 05:13 am</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>CSEEXPO-2026-0002</v>
-      </c>
-      <c r="B5" t="str">
-        <v>PulseGuard</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Diya Patel</v>
-      </c>
-      <c r="D5" t="str">
-        <v>+919876543211</v>
-      </c>
-      <c r="E5" t="str">
-        <v>diya.patel@gmail.com</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Non-Invasive Wearable Cardiac &amp; Hypoxia Alert Band</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Healthcare</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Rural patients experiencing arrhythmia and nocturnal hypoxia often face delayed emergency response due to absence of affordable continuous telemetry.</v>
-      </c>
-      <c r="I5" t="str">
-        <v>A wristband running lightweight tinyML for anomaly classification in PPG waveform with GSM-assisted SOS beaconing.</v>
-      </c>
-      <c r="J5" t="str">
-        <v>React, FastAPI, Scikit-learn, WebSockets, Supabase</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Raspberry Pi Pico W, MAX30102 PPG Sensor, AD8232 ECG Sensor, SIM800L GSM Module, 0.96 OLED Display</v>
-      </c>
-      <c r="L5" t="str">
-        <v>Continuous 24-hr vitals monitoring with sub-3 second emergency trigger.</v>
-      </c>
-      <c r="M5" t="str">
-        <v>Diya Patel</v>
-      </c>
-      <c r="N5" t="str">
-        <v>4th Year</v>
-      </c>
-      <c r="O5" t="str">
-        <v>B</v>
-      </c>
-      <c r="P5" t="str">
-        <v>Eshwar Rao</v>
-      </c>
-      <c r="Q5" t="str">
-        <v>4th Year</v>
-      </c>
-      <c r="R5" t="str">
-        <v>B</v>
-      </c>
-      <c r="S5" t="str">
-        <v>Farhan Khan</v>
-      </c>
-      <c r="T5" t="str">
-        <v>4th Year</v>
-      </c>
-      <c r="U5" t="str">
-        <v>C</v>
-      </c>
-      <c r="V5" t="str">
-        <v/>
-      </c>
-      <c r="W5" t="str">
-        <v/>
-      </c>
-      <c r="X5" t="str">
-        <v/>
-      </c>
-      <c r="Y5" t="str">
-        <v/>
-      </c>
-      <c r="Z5" t="str">
-        <v/>
-      </c>
-      <c r="AA5" t="str">
-        <v/>
-      </c>
-      <c r="AB5" t="str">
-        <v/>
-      </c>
-      <c r="AC5" t="str">
-        <v/>
-      </c>
-      <c r="AD5" t="str">
-        <v/>
-      </c>
-      <c r="AE5" t="str">
-        <v>SHORTLISTED</v>
-      </c>
-      <c r="AF5" t="str">
-        <v>25 Sept 2026, 05:13 am</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>CSEEXPO-2026-0005</v>
-      </c>
-      <c r="B6" t="str">
-        <v>SafeStream AI</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Vikram Singh</v>
-      </c>
-      <c r="D6" t="str">
-        <v>+919876543214</v>
-      </c>
-      <c r="E6" t="str">
-        <v>vikram.singh@gmail.com</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Vision-Based Industrial Machine Safety Interlock</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Artificial Intelligence</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Accidents at mechanical presses occur when operators bypass safety light curtains during shifts.</v>
-      </c>
-      <c r="I6" t="str">
-        <v>Stereo-vision edge module tracking operator hands, predicting trajectory, and triggering electronic emergency brakes in 40ms.</v>
-      </c>
-      <c r="J6" t="str">
-        <v>C++, OpenCV, CUDA, TensorRT, Electron Dashboard</v>
-      </c>
-      <c r="K6" t="str">
-        <v>NVIDIA Jetson Orin Nano, Dual Global Shutter CSI Cameras, Optocoupler Relay Isolation Board</v>
-      </c>
-      <c r="L6" t="str">
-        <v>Zero false negatives in safety hazard classification.</v>
-      </c>
-      <c r="M6" t="str">
-        <v>Vikram Singh</v>
-      </c>
-      <c r="N6" t="str">
-        <v>3rd Year</v>
-      </c>
-      <c r="O6" t="str">
-        <v>B</v>
-      </c>
-      <c r="P6" t="str">
-        <v>Jaya Prakash</v>
-      </c>
-      <c r="Q6" t="str">
-        <v>3rd Year</v>
-      </c>
-      <c r="R6" t="str">
-        <v>B</v>
-      </c>
-      <c r="S6" t="str">
-        <v>Karan Malhotra</v>
-      </c>
-      <c r="T6" t="str">
-        <v>3rd Year</v>
-      </c>
-      <c r="U6" t="str">
-        <v>C</v>
-      </c>
-      <c r="V6" t="str">
-        <v/>
-      </c>
-      <c r="W6" t="str">
-        <v/>
-      </c>
-      <c r="X6" t="str">
-        <v/>
-      </c>
-      <c r="Y6" t="str">
-        <v/>
-      </c>
-      <c r="Z6" t="str">
-        <v/>
-      </c>
-      <c r="AA6" t="str">
-        <v/>
-      </c>
-      <c r="AB6" t="str">
-        <v/>
-      </c>
-      <c r="AC6" t="str">
-        <v/>
-      </c>
-      <c r="AD6" t="str">
-        <v/>
-      </c>
-      <c r="AE6" t="str">
-        <v>SHORTLISTED</v>
-      </c>
-      <c r="AF6" t="str">
-        <v>24 Sept 2026, 05:13 am</v>
+        <v>2026-09-23T23:59:34.774Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AF6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: configure utility template expo_team_update for admin broadcast and sync latest 7 live teams
</commit_message>
<xml_diff>
--- a/data/teams_export.xlsx
+++ b/data/teams_export.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF4"/>
+  <dimension ref="A1:AF8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -497,60 +497,110 @@
         <v>Submitted Date</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>CSEEXPO-2026-0003</v>
+        <v>CSEEXPO-2026-0001</v>
       </c>
       <c r="B2" t="str">
-        <v>Techora</v>
+        <v>karthi</v>
       </c>
       <c r="C2" t="str">
-        <v>Madhu Sree</v>
+        <v>Karnexha Offc</v>
       </c>
       <c r="D2" t="str">
-        <v>+919025896972</v>
+        <v>+918778606059</v>
       </c>
       <c r="E2" t="str">
-        <v>madhusreemanokaran@gmail.com</v>
+        <v>karnexhaoffc@gmail.com</v>
       </c>
       <c r="F2" t="str">
-        <v>Gridguard Ai</v>
+        <v>test11111</v>
       </c>
       <c r="G2" t="str">
-        <v>Artificial Intelligence</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Gridguard Ai in Lt line and automatic emergency shutdown</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Using Sensors like temperature,voltage we can find the status of Lt line</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Python Flask</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Lora Module</v>
+        <v>Agriculture</v>
+      </c>
+      <c r="H2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Team &amp; Project Specifications
+Enter your team identity, problem theme, and hardware/software technical architecture.
+Software + Hardware
+Team Name*
+e.g. AgriSense IoT
+Team Leader Full Name*</v>
+      </c>
+      <c r="I2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Team &amp; Project Specifications
+Enter your team identity, problem theme, and hardware/software technical architecture.
+Software + Hardware
+Team Name*
+e.g. AgriSense IoT
+Team Leader Full Name*
+Step 1: Team &amp; Project Specifications
+Enter your team identity, problem theme, and hardware/software technical architecture.
+Software + Hardware
+Team Name*
+e.g. AgriSense IoT
+Team Leader Full Name*</v>
+      </c>
+      <c r="J2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Team &amp; Project Specifications
+Enter your team identity, problem theme, and hardware/software technical architecture.
+Software + Hardware
+Team Name*
+e.g. AgriSense IoT
+Team Leader Full Name*
+Step 1: Team &amp; Project Specifications
+Enter your team identity, problem theme, and hardware/software technical architecture.
+Software + Hardware
+Team Name*
+e.g. AgriSense IoT
+Team Leader Full Name*
+Step 1: Team &amp; Project Specifications
+Enter your team identity, problem theme, and hardware/software technical architecture.
+Software + Hardware
+Team Name*
+e.g. AgriSense IoT
+Team Leader Full Name*</v>
+      </c>
+      <c r="K2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Team &amp; Project Specifications
+Enter your team identity, problem theme, and hardware/software technical architecture.
+Software + Hardware
+Team Name*
+e.g. AgriSense IoT
+Team Leader Full Name*
+Step 1: Team &amp; Project Specifications
+Enter your team identity, problem theme, and hardware/software technical architecture.
+Software + Hardware
+Team Name*
+e.g. AgriSense IoT
+Team Leader Full Name*
+Step 1: Team &amp; Project Specifications
+Enter your team identity, problem theme, and hardware/software technical architecture.
+Software + Hardware
+Team Name*
+e.g. AgriSense IoT
+Team Leader Full Name*</v>
       </c>
       <c r="L2" t="str">
         <v/>
       </c>
       <c r="M2" t="str">
-        <v>Madhu Sree</v>
+        <v>Karnexha Offc</v>
       </c>
       <c r="N2" t="str">
-        <v>3rd Year</v>
+        <v>1st Year</v>
       </c>
       <c r="O2" t="str">
-        <v>B</v>
+        <v>G</v>
       </c>
       <c r="P2" t="str">
-        <v>Gracy</v>
+        <v>karthi</v>
       </c>
       <c r="Q2" t="str">
-        <v>3rd Year</v>
+        <v>1st Year</v>
       </c>
       <c r="R2" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="S2" t="str">
         <v/>
@@ -592,90 +642,90 @@
         <v>SUBMITTED</v>
       </c>
       <c r="AF2" t="str">
-        <v>2026-09-29T00:23:54.151Z</v>
+        <v>2026-09-29T06:33:07.847Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>CSEEXPO-2026-0003</v>
+        <v>CSEEXPO-2026-0005</v>
       </c>
       <c r="B3" t="str">
-        <v>NeuroBraille</v>
+        <v>SS tech</v>
       </c>
       <c r="C3" t="str">
-        <v>Rohan Verma</v>
+        <v>Sadha Sivam</v>
       </c>
       <c r="D3" t="str">
-        <v>+919876543212</v>
+        <v>+916379261134</v>
       </c>
       <c r="E3" t="str">
-        <v>rohan.verma@gmail.com</v>
+        <v>sadhasivam17092008@gmail.com</v>
       </c>
       <c r="F3" t="str">
-        <v>Dynamic Refreshable Braille Slate with Voice OCR</v>
+        <v>Automatic plant watering system</v>
       </c>
       <c r="G3" t="str">
-        <v>Education</v>
+        <v>Agriculture</v>
       </c>
       <c r="H3" t="str">
-        <v>Commercial refreshable Braille displays cost upwards of $2,000, rendering them inaccessible to 95% of visually impaired students.</v>
+        <v>Plants need regular watering for healthy growth, but people may forget to water them due to busy schedules or being away from home. Manual watering can also result in overwatering or underwatering. This may affect the health and growth of plants and waste water. Therefore, an automatic system is needed to monitor soil moisture and provide the required amount of water whenever the soil becomes dry.</v>
       </c>
       <c r="I3" t="str">
-        <v>A low-cost 32-cell electromagnetic Braille display combined with an overhead camera that performs optical character recognition.</v>
+        <v>The proposed system is an automatic plant watering system using an Arduino and a soil moisture sensor. The sensor continuously monitors the moisture level of the soil. When the soil becomes too dry, the Arduino automatically activates a water pump to supply water to the plant. Once the soil reaches the required moisture level, the pump is turned off automatically. This reduces the need for manual watering and helps prevent water wastage.</v>
       </c>
       <c r="J3" t="str">
-        <v>Python OpenCV, Tesseract OCR, PyTorch, Node.js API</v>
+        <v>Arduino IDE(Integrated Development Environment)</v>
       </c>
       <c r="K3" t="str">
-        <v>STM32 Nucleo Board, 192 Micro-solenoid Actuators, OV5640 Camera Module, Bone-conduction Audio Transducer</v>
+        <v>Adriuno nano,Soil moisture sensor module,0.96 inch display,water pump.</v>
       </c>
       <c r="L3" t="str">
-        <v>Affordable dynamic Braille reading device manufactured under INR 4,500.</v>
+        <v/>
       </c>
       <c r="M3" t="str">
-        <v>Rohan Verma</v>
+        <v>Sadha Sivam</v>
       </c>
       <c r="N3" t="str">
-        <v>2nd Year</v>
+        <v>1st Year</v>
       </c>
       <c r="O3" t="str">
-        <v>C</v>
+        <v>F</v>
       </c>
       <c r="P3" t="str">
-        <v>Gaurav Mehta</v>
+        <v>Sree Hari</v>
       </c>
       <c r="Q3" t="str">
-        <v>2nd Year</v>
+        <v>1st Year</v>
       </c>
       <c r="R3" t="str">
-        <v>C</v>
+        <v>F</v>
       </c>
       <c r="S3" t="str">
-        <v>Harini Swaminathan</v>
+        <v>Sibidharan</v>
       </c>
       <c r="T3" t="str">
-        <v>2nd Year</v>
+        <v>1st Year</v>
       </c>
       <c r="U3" t="str">
-        <v>D</v>
+        <v>F</v>
       </c>
       <c r="V3" t="str">
-        <v/>
+        <v>Sri Sanjai Raghav</v>
       </c>
       <c r="W3" t="str">
-        <v/>
+        <v>1st Year</v>
       </c>
       <c r="X3" t="str">
-        <v/>
+        <v>F</v>
       </c>
       <c r="Y3" t="str">
-        <v/>
+        <v>Salman Faris</v>
       </c>
       <c r="Z3" t="str">
-        <v/>
+        <v>1st Year</v>
       </c>
       <c r="AA3" t="str">
-        <v/>
+        <v>F</v>
       </c>
       <c r="AB3" t="str">
         <v/>
@@ -687,51 +737,51 @@
         <v/>
       </c>
       <c r="AE3" t="str">
-        <v>REJECTED</v>
+        <v>SUBMITTED</v>
       </c>
       <c r="AF3" t="str">
-        <v>2026-09-26T23:59:34.774Z</v>
+        <v>2026-09-30T12:34:49.807Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>CSEEXPO-2026-0005</v>
+        <v>CSEEXPO-2026-0007</v>
       </c>
       <c r="B4" t="str">
-        <v>SafeStream AI</v>
+        <v>Mednova</v>
       </c>
       <c r="C4" t="str">
-        <v>Vikram Singh</v>
+        <v>Madhu Sree</v>
       </c>
       <c r="D4" t="str">
-        <v>+919876543214</v>
+        <v>+919025896972</v>
       </c>
       <c r="E4" t="str">
-        <v>vikram.singh@gmail.com</v>
+        <v>madhusreemanokaran@gmail.com</v>
       </c>
       <c r="F4" t="str">
-        <v>Vision-Based Industrial Machine Safety Interlock</v>
+        <v>Mednova</v>
       </c>
       <c r="G4" t="str">
-        <v>Artificial Intelligence</v>
+        <v>Healthcare</v>
       </c>
       <c r="H4" t="str">
-        <v>Accidents at mechanical presses occur when operators bypass safety light curtains during shifts.</v>
+        <v>Mannual medical submission reports</v>
       </c>
       <c r="I4" t="str">
-        <v>Stereo-vision edge module tracking operator hands, predicting trajectory, and triggering electronic emergency brakes in 40ms.</v>
+        <v>Using Ai for medical reports which is useful for patients</v>
       </c>
       <c r="J4" t="str">
-        <v>C++, OpenCV, CUDA, TensorRT, Electron Dashboard</v>
+        <v>Next.js</v>
       </c>
       <c r="K4" t="str">
-        <v>NVIDIA Jetson Orin Nano, Dual Global Shutter CSI Cameras, Optocoupler Relay Isolation Board</v>
+        <v>LoraModule</v>
       </c>
       <c r="L4" t="str">
-        <v>Zero false negatives in safety hazard classification.</v>
+        <v/>
       </c>
       <c r="M4" t="str">
-        <v>Vikram Singh</v>
+        <v>Madhu Sree</v>
       </c>
       <c r="N4" t="str">
         <v>3rd Year</v>
@@ -740,7 +790,7 @@
         <v>B</v>
       </c>
       <c r="P4" t="str">
-        <v>Jaya Prakash</v>
+        <v>Gracy</v>
       </c>
       <c r="Q4" t="str">
         <v>3rd Year</v>
@@ -749,13 +799,13 @@
         <v>B</v>
       </c>
       <c r="S4" t="str">
-        <v>Karan Malhotra</v>
+        <v>Maragatham</v>
       </c>
       <c r="T4" t="str">
         <v>3rd Year</v>
       </c>
       <c r="U4" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="V4" t="str">
         <v/>
@@ -785,15 +835,438 @@
         <v/>
       </c>
       <c r="AE4" t="str">
-        <v>SHORTLISTED</v>
+        <v>SUBMITTED</v>
       </c>
       <c r="AF4" t="str">
-        <v>2026-09-23T23:59:34.774Z</v>
+        <v>2026-09-30T14:39:24.447Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>CSEEXPO-2026-0006</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Cipher</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Rishid S</v>
+      </c>
+      <c r="D5" t="str">
+        <v>+919443588231</v>
+      </c>
+      <c r="E5" t="str">
+        <v>rishids123@gmail.com</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Smart Farm Guard: Ultrasonic-Based Stray Animal Intrusion Detection and Alert System</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Agriculture</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Farmers living near forest edges and rural areas lose a significant part of their crops to stray animals such as wild boars, cattle and elephants entering fields, mostly at night. Guarding the fields manually is tiring, unsafe and not affordable for small farmers, and solutions like electric fencing are expensive and can be dangerous to both animals and people. There is a need for a low-cost system that can detect an intrusion at a field entry point and alert the farmer immediately, so that action can be taken before the crop is damaged.</v>
+      </c>
+      <c r="I5" t="str">
+        <v>The system is built around an ESP32 microcontroller connected to an HC-SR04 ultrasonic sensor placed at a field entry point such as a gate or a gap in the fence. The sensor continuously measures the distance of objects in front of it. When an object comes closer than a preset threshold for several consecutive readings, the ESP32 treats it as an intrusion and immediately activates a buzzer and a flashing LED to scare the animal away. Each event is logged with a timestamp, and the farmer can view live distance readings and the intrusion log on a web dashboard hosted by the ESP32 over Wi-Fi.</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Arduino IDE, Embedded C/C++, ESP32 Arduino Core, WebServer library (ESP32 as a Wi-Fi web server), HTML/CSS for the dashboard page</v>
+      </c>
+      <c r="K5" t="str">
+        <v>ESP32 DevKit (microcontroller with Wi-Fi), HC-SR04 Ultrasonic Sensor, Active Buzzer, LED with 220Ω resistor, 1kΩ and 2kΩ resistors (voltage divider for the Echo pin), Breadboard, Jumper Wires, USB Cable / 5V Power Bank</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v>Rishid S</v>
+      </c>
+      <c r="N5" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="O5" t="str">
+        <v>E</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Ritesh</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="R5" t="str">
+        <v>E</v>
+      </c>
+      <c r="S5" t="str">
+        <v>Pranesh T</v>
+      </c>
+      <c r="T5" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="U5" t="str">
+        <v>E</v>
+      </c>
+      <c r="V5" t="str">
+        <v>Pranesh P</v>
+      </c>
+      <c r="W5" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="X5" t="str">
+        <v>E</v>
+      </c>
+      <c r="Y5" t="str">
+        <v>Praveen M</v>
+      </c>
+      <c r="Z5" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="AA5" t="str">
+        <v>E</v>
+      </c>
+      <c r="AB5" t="str">
+        <v>Rishindhar</v>
+      </c>
+      <c r="AC5" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="AD5" t="str">
+        <v>E</v>
+      </c>
+      <c r="AE5" t="str">
+        <v>SUBMITTED</v>
+      </c>
+      <c r="AF5" t="str">
+        <v>2026-09-30T13:51:16.672Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>CSEEXPO-2026-0003</v>
+      </c>
+      <c r="B6" t="str">
+        <v>NextGenz</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Bhuvana A</v>
+      </c>
+      <c r="D6" t="str">
+        <v>+919750551880</v>
+      </c>
+      <c r="E6" t="str">
+        <v>bhuvibhuvana1106@gmail.com</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Life raft AI</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Education</v>
+      </c>
+      <c r="H6" t="str">
+        <v>After completing 12th grade, many students feel confused about choosing the right course, career, or future path. They may not know their strengths, interests, or the skills needed for different careers. At the same time, students get fewer opportunities to practice real-life skills like decision-making, problem-solving, teamwork, and financial management. LifeCraft AI helps solve this problem through an interactive game where students explore different situations, make decisions, understand the results, and discover their skills and interests in an engaging way</v>
+      </c>
+      <c r="I6" t="str">
+        <v>LifeCraft AI is a web-based game that gives students different real-life situations. Students make decisions and see the results of their choices. The game has different levels, challenges, and stories. Their skills such as problem-solving, decision-making, creativity, teamwork, and financial skills increase as they complete the levels. An AI assistant called LUMA gives hints and guidance during the game. After completing all levels, students can unlock their certificate.</v>
+      </c>
+      <c r="J6" t="str">
+        <v>React.js, TypeScript, HTML, CSS, Node.js, AI/LLM API, Database, REST API</v>
+      </c>
+      <c r="K6" t="str">
+        <v>No hardware or sensors is required</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v>Bhuvana A</v>
+      </c>
+      <c r="N6" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="O6" t="str">
+        <v>A</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Anitha C</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="R6" t="str">
+        <v>A</v>
+      </c>
+      <c r="S6" t="str">
+        <v>Dharshini B</v>
+      </c>
+      <c r="T6" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="U6" t="str">
+        <v>A</v>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v/>
+      </c>
+      <c r="Y6" t="str">
+        <v/>
+      </c>
+      <c r="Z6" t="str">
+        <v/>
+      </c>
+      <c r="AA6" t="str">
+        <v/>
+      </c>
+      <c r="AB6" t="str">
+        <v/>
+      </c>
+      <c r="AC6" t="str">
+        <v/>
+      </c>
+      <c r="AD6" t="str">
+        <v/>
+      </c>
+      <c r="AE6" t="str">
+        <v>UNDER_REVIEW</v>
+      </c>
+      <c r="AF6" t="str">
+        <v>2026-09-29T15:56:38.045Z</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>CSEEXPO-2026-0006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Titanic six</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Yazhini Athishkumar</v>
+      </c>
+      <c r="D7" t="str">
+        <v>+919342356256</v>
+      </c>
+      <c r="E7" t="str">
+        <v>yazhiniathish@gmail.com</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Fishermen border alert</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Social Impact</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Small-scale fishermen often cross invisible international maritime boundaries by accident because their boats lack an affordable way to track their position, leading to arrests, seized boats, and lost livelihoods.</v>
+      </c>
+      <c r="I7" t="str">
+        <v>This project aims to build a low-cost GPS-based device that warns fishermen with a buzzer and lights as they near the boundary and sends their live location to family and authorities.</v>
+      </c>
+      <c r="J7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Arduino IDE (C/C++),
+TinyGPS++,
+Geofencing logic (Haversine formula),
+Firebase etc</v>
+      </c>
+      <c r="K7" t="str" xml:space="preserve">
+        <v xml:space="preserve">ESP32,
+GPS module (NEO-6M),
+GSM module (SIM800L),
+Buzzer + LEDs etc</v>
+      </c>
+      <c r="L7" t="str">
+        <v>A low-cost device that gives fishermen early border warnings and lets families track them, reducing accidental arrests, protecting livelihoods, and improving safety at sea.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Yazhini Athishkumar</v>
+      </c>
+      <c r="N7" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="O7" t="str">
+        <v>G</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Trinitta Rani.A</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="R7" t="str">
+        <v>G</v>
+      </c>
+      <c r="S7" t="str">
+        <v>Vijaya Dharshini.N</v>
+      </c>
+      <c r="T7" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="U7" t="str">
+        <v>G</v>
+      </c>
+      <c r="V7" t="str">
+        <v>Thanisha Poornima .S</v>
+      </c>
+      <c r="W7" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="X7" t="str">
+        <v>G</v>
+      </c>
+      <c r="Y7" t="str">
+        <v>Thabiksha.V</v>
+      </c>
+      <c r="Z7" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="AA7" t="str">
+        <v>G</v>
+      </c>
+      <c r="AB7" t="str">
+        <v>Vaishnavi Devi.S</v>
+      </c>
+      <c r="AC7" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="AD7" t="str">
+        <v>G</v>
+      </c>
+      <c r="AE7" t="str">
+        <v>SUBMITTED</v>
+      </c>
+      <c r="AF7" t="str">
+        <v>2026-09-30T14:39:06.288Z</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>CSEEXPO-2026-0004</v>
+      </c>
+      <c r="B8" t="str">
+        <v>INVICTUS</v>
+      </c>
+      <c r="C8" t="str">
+        <v>JAIKAILAS GK</v>
+      </c>
+      <c r="D8" t="str">
+        <v>+919488779796</v>
+      </c>
+      <c r="E8" t="str">
+        <v>gkkailas10@gmail.com</v>
+      </c>
+      <c r="F8" t="str">
+        <v>GEOSHIELD -- TOURIST SAFETY SYSTEM</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Social Impact</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Tourists traveling in unfamiliar locations often face safety challenges such as entering unsafe zones, getting lost, language barriers, delayed emergency assistance, and lack of real-time information about potential threats. Existing safety solutions primarily react after an incident occurs rather than preventing risks beforehand. This can lead to increased response times and reduced traveler confidence, especially in remote or crowded tourist destinations.</v>
+      </c>
+      <c r="I8" t="str">
+        <v>GEOSHIELD is an AI-powered Tourist Safety Application designed to provide proactive protection and rapid emergency response for travelers. The system combines real-time GPS tracking, wearable IoT devices, predictive risk analysis, geofencing technology, and instant SOS communication to continuously monitor tourist safety. By detecting potential threats, sending early warnings, and automatically coordinating with emergency services, GEOSHIELD helps ensure safer travel experiences while reducing response times during critical situations.</v>
+      </c>
+      <c r="J8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Front-End &amp; Mobile Development
+React.js – User interface development
+TypeScript – Type-safe application development
+Vite – Fast build and development environment
+Tailwind CSS – Responsive and modern UI design
+Back-End &amp; Cloud Services
+FastAPI (Python) – High-performance REST API development
+Node.js – Real-time backend services and integrations
+Render Cloud Platform – Application deployment and hosting
+Artificial Intelligence &amp; Machine Learning
+Groq API (Llama 3.3) – Threat analysis, emergency message processing, and decision support
+YOLOv8 – Safety object detection and environmental hazard identification
+Predictive Analytics Models – Risk prediction and tourist safety assessment
+Blockchain &amp; IoT
+Hyperledger Fabric – Secure and tamper-proof incident logging
+LoRaWAN – Long-range emergency communication
+GSM/GPS Modules – Real-time location tracking and SOS transmission
+Wearable IoT Devices – Panic button and tourist monitoring
+Database
+MySQL 8.0 – Storage of user, location, incident, alert, and prediction data</v>
+      </c>
+      <c r="K8" t="str" xml:space="preserve">
+        <v xml:space="preserve">📍 GPS Sensor – Tourist location track panna
+📐 6-Axis IMU / Accelerometer (MPU6050) – Slip, fall, sudden movement detect panna
+🌡️ Barometric Pressure Sensor (BMP390) – Altitude &amp; sudden pressure changes detect panna
+❤️ Heart Rate Sensor (MAX30102) – Heart-rate changes monitor panna
+💧 Temperature &amp; Humidity Sensor (SHT30) – Weather/environment condition monitor panna
+🌊 Water Detection Sensor – Water/flash-flood exposure detect panna
+ soil sensors --  this only not insert in the bracelet</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Improves tourist safety and confidence through real-time monitoring, alerts, and rapid emergency response. Supports authorities with accurate location tracking and faster rescue coordination during emergencies. Promotes tourism growth while enabling safe and sustainable management of environmentally sensitive areas.</v>
+      </c>
+      <c r="M8" t="str">
+        <v>JAIKAILAS GK</v>
+      </c>
+      <c r="N8" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="O8" t="str">
+        <v>B</v>
+      </c>
+      <c r="P8" t="str">
+        <v>JOTHI DHARSHAN K</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="R8" t="str">
+        <v>B</v>
+      </c>
+      <c r="S8" t="str">
+        <v>KINGSTON DANIEL S</v>
+      </c>
+      <c r="T8" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="U8" t="str">
+        <v>B</v>
+      </c>
+      <c r="V8" t="str">
+        <v>LOKENETHREN P</v>
+      </c>
+      <c r="W8" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="X8" t="str">
+        <v>B</v>
+      </c>
+      <c r="Y8" t="str">
+        <v>KRITHIK B</v>
+      </c>
+      <c r="Z8" t="str">
+        <v>2nd Year</v>
+      </c>
+      <c r="AA8" t="str">
+        <v>B</v>
+      </c>
+      <c r="AB8" t="str">
+        <v/>
+      </c>
+      <c r="AC8" t="str">
+        <v/>
+      </c>
+      <c r="AD8" t="str">
+        <v/>
+      </c>
+      <c r="AE8" t="str">
+        <v>SUBMITTED</v>
+      </c>
+      <c r="AF8" t="str">
+        <v>2026-09-30T05:20:45.888Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AF4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>